<commit_message>
split outcome notes into comments and error codes
</commit_message>
<xml_diff>
--- a/data/source/i1_raw_data.xlsx
+++ b/data/source/i1_raw_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djo/dev/au/au_diss/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djo/dev/au/au_diss/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7DDC03-7A7D-5C46-B8BC-422113988FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3EA9D7-713F-504A-AF1E-F48398DFE83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23040" yWindow="500" windowWidth="23040" windowHeight="25420" activeTab="7" xr2:uid="{9D3AC3E5-42CD-5B4C-9A6D-E91B574DC308}"/>
+    <workbookView xWindow="20040" yWindow="500" windowWidth="40120" windowHeight="33340" activeTab="7" xr2:uid="{9D3AC3E5-42CD-5B4C-9A6D-E91B574DC308}"/>
   </bookViews>
   <sheets>
     <sheet name="DEMO" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1609" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1609" uniqueCount="253">
   <si>
     <t>Participant</t>
   </si>
@@ -459,9 +459,6 @@
     <t>Flag</t>
   </si>
   <si>
-    <t>67 and 59 flipped, L and R</t>
-  </si>
-  <si>
     <t>did not correct errors learned in p1</t>
   </si>
   <si>
@@ -477,9 +474,6 @@
     <t>mostly memorized</t>
   </si>
   <si>
-    <t>didn't use instructions; incomplete, one piece missing (88L)</t>
-  </si>
-  <si>
     <t>no PWI?</t>
   </si>
   <si>
@@ -489,13 +483,7 @@
     <t>during practice experienced issues with selection and interface; long sleeves interfered with hand recognition; model tracking issues; most errors incorrectly recorded in DCS</t>
   </si>
   <si>
-    <t>front 67 LR misplaced</t>
-  </si>
-  <si>
     <t>DCS shows 59/67 swapped but correct as pictured</t>
-  </si>
-  <si>
-    <t>F67LRP; S1 all 5 parts incorrecly located, one added 75</t>
   </si>
   <si>
     <t>F59LRS (2), F67LRP (2), R59LRPR (2+2), R74LP (1), R74RS (1), R1RS (1)</t>
@@ -577,9 +565,6 @@
   </si>
   <si>
     <t>F88LRP (2)</t>
-  </si>
-  <si>
-    <t>F88LRP (2); F24 (cross-member) incorrectly reinstalled</t>
   </si>
   <si>
     <t>same error as in learning</t>
@@ -678,9 +663,6 @@
     <t>R1AP (3)</t>
   </si>
   <si>
-    <t>R1AP (3), F74LRS (2) - added black 2x2s behind hinges</t>
-  </si>
-  <si>
     <t>R59LRP (2), R74LRP (2), R75CP (1)</t>
   </si>
   <si>
@@ -691,9 +673,6 @@
   </si>
   <si>
     <t>F59LRS (2)</t>
-  </si>
-  <si>
-    <t>R1LS (2) - two duplicate pieces added</t>
   </si>
   <si>
     <t>F59LRS (2), F67LRP (2), R59LRP (2), R74LRP (2), R75CP (1)</t>
@@ -712,9 +691,6 @@
   </si>
   <si>
     <t>car axle stuck in fixture, corrected</t>
-  </si>
-  <si>
-    <t>F88LRP (2); corrected 88 rotation not placement</t>
   </si>
   <si>
     <t>didn't start next car</t>
@@ -765,12 +741,6 @@
     <t>F59LRS (2); F67LRS (2), F88LRR (2), F88LRP (2)</t>
   </si>
   <si>
-    <t>R74LRP (2); also missing part 89R from before</t>
-  </si>
-  <si>
-    <t>R3RS (1); missing part 89R from before (no error)</t>
-  </si>
-  <si>
     <t>R75CP (1)</t>
   </si>
   <si>
@@ -807,10 +777,34 @@
     <t>p88 detached while moving to green bin at time</t>
   </si>
   <si>
-    <t>R59LRP (2), R74LRP (2); r65 slightly offset (no error)</t>
+    <t>learning is not just about reps</t>
   </si>
   <si>
-    <t>learning is not just about reps</t>
+    <t>F67LRP (2), R59LRP (2), R74LRP (2), R75CP (1), R75CS (1)</t>
+  </si>
+  <si>
+    <t>R1AP (3), F74LRS (2) :: added black 2x2s behind hinges</t>
+  </si>
+  <si>
+    <t>R1LS (2) :: two duplicate pieces added</t>
+  </si>
+  <si>
+    <t>F88LRP (2) :: corrected 88 rotation not placement</t>
+  </si>
+  <si>
+    <t>F88LRP (2) :: F24 (cross-member) incorrectly reinstalled</t>
+  </si>
+  <si>
+    <t>R3RS (1) :: missing part 89R from before (no error)</t>
+  </si>
+  <si>
+    <t>R74LRP (2) :: also missing part 89R from before</t>
+  </si>
+  <si>
+    <t>R59LRP (2), R74LRP (2) :: r65 slightly offset (no error)</t>
+  </si>
+  <si>
+    <t>F88LS (1) :: didn't use instructions, incomplete, one piece missing</t>
   </si>
 </sst>
 </file>
@@ -26937,7 +26931,7 @@
         <v>131</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="K1" s="11" t="s">
         <v>60</v>
@@ -26989,10 +26983,9 @@
       </c>
       <c r="I3" s="13"/>
       <c r="J3" s="13"/>
-      <c r="K3" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="L3" s="12"/>
+      <c r="K3" s="12" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="13">
@@ -27010,8 +27003,8 @@
       <c r="H4" s="13">
         <v>4</v>
       </c>
-      <c r="K4" s="14" t="s">
-        <v>137</v>
+      <c r="K4" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -27049,8 +27042,8 @@
       <c r="H6" s="13">
         <v>4</v>
       </c>
-      <c r="K6" s="14" t="s">
-        <v>137</v>
+      <c r="K6" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -27070,8 +27063,8 @@
       <c r="H7" s="13">
         <v>4</v>
       </c>
-      <c r="K7" s="14" t="s">
-        <v>137</v>
+      <c r="K7" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -27090,8 +27083,8 @@
       <c r="H8" s="13">
         <v>4</v>
       </c>
-      <c r="K8" s="14" t="s">
-        <v>137</v>
+      <c r="K8" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
@@ -27129,8 +27122,8 @@
       <c r="H10" s="13">
         <v>4</v>
       </c>
-      <c r="K10" s="14" t="s">
-        <v>137</v>
+      <c r="K10" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -27150,8 +27143,8 @@
       <c r="H11" s="13">
         <v>4</v>
       </c>
-      <c r="K11" s="14" t="s">
-        <v>137</v>
+      <c r="K11" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -27168,7 +27161,7 @@
         <v>41</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -27187,8 +27180,8 @@
       <c r="H13" s="13">
         <v>4</v>
       </c>
-      <c r="K13" s="14" t="s">
-        <v>137</v>
+      <c r="K13" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
@@ -27207,8 +27200,8 @@
       <c r="H14" s="13">
         <v>4</v>
       </c>
-      <c r="K14" s="14" t="s">
-        <v>137</v>
+      <c r="K14" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
@@ -27227,8 +27220,8 @@
       <c r="H15" s="13">
         <v>4</v>
       </c>
-      <c r="K15" s="14" t="s">
-        <v>137</v>
+      <c r="K15" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
@@ -27247,8 +27240,8 @@
       <c r="H16" s="13">
         <v>4</v>
       </c>
-      <c r="K16" s="14" t="s">
-        <v>137</v>
+      <c r="K16" s="12" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
@@ -27265,7 +27258,7 @@
         <v>41</v>
       </c>
       <c r="K17" s="14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -27310,7 +27303,7 @@
         <v>0</v>
       </c>
       <c r="K20" s="14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -27327,7 +27320,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -27355,7 +27348,7 @@
         <v>6</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
@@ -27364,7 +27357,7 @@
         <v>15</v>
       </c>
       <c r="K23" t="s">
-        <v>143</v>
+        <v>252</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
@@ -27381,7 +27374,7 @@
         <v>41</v>
       </c>
       <c r="K24" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -27398,7 +27391,7 @@
         <v>0</v>
       </c>
       <c r="K25" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
@@ -27429,7 +27422,7 @@
         <v>0</v>
       </c>
       <c r="K27" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -27460,7 +27453,7 @@
         <v>41</v>
       </c>
       <c r="K29" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
@@ -27480,7 +27473,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
@@ -27500,7 +27493,7 @@
         <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>147</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -27523,7 +27516,7 @@
         <v>7</v>
       </c>
       <c r="K32" t="s">
-        <v>149</v>
+        <v>244</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
@@ -27540,7 +27533,7 @@
         <v>41</v>
       </c>
       <c r="K33" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -27566,7 +27559,7 @@
         <v>2</v>
       </c>
       <c r="K34" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
@@ -27592,7 +27585,7 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
@@ -27615,7 +27608,7 @@
         <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -27638,7 +27631,7 @@
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -27655,7 +27648,7 @@
         <v>41</v>
       </c>
       <c r="K38" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -27711,7 +27704,7 @@
         <v>4</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F42" s="1">
         <v>0</v>
@@ -27720,7 +27713,7 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
@@ -27737,7 +27730,7 @@
         <v>41</v>
       </c>
       <c r="K43" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -27810,7 +27803,7 @@
         <v>41</v>
       </c>
       <c r="K48" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
@@ -27866,7 +27859,7 @@
         <v>4</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F52" s="1">
         <v>0</v>
@@ -27875,7 +27868,7 @@
         <v>11</v>
       </c>
       <c r="K52" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
@@ -27892,7 +27885,7 @@
         <v>41</v>
       </c>
       <c r="K53" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
@@ -27965,7 +27958,7 @@
         <v>41</v>
       </c>
       <c r="K58" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
@@ -27985,7 +27978,7 @@
         <v>1</v>
       </c>
       <c r="K59" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
@@ -28005,7 +27998,7 @@
         <v>1</v>
       </c>
       <c r="K60" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
@@ -28092,7 +28085,7 @@
         <v>41</v>
       </c>
       <c r="K66" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
@@ -28154,7 +28147,7 @@
         <v>0</v>
       </c>
       <c r="K70" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
@@ -28171,7 +28164,7 @@
         <v>41</v>
       </c>
       <c r="K71" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
@@ -28191,7 +28184,7 @@
         <v>7</v>
       </c>
       <c r="K72" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
@@ -28211,7 +28204,7 @@
         <v>7</v>
       </c>
       <c r="K73" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
@@ -28231,7 +28224,7 @@
         <v>7</v>
       </c>
       <c r="K74" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
@@ -28251,7 +28244,7 @@
         <v>7</v>
       </c>
       <c r="K75" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
@@ -28268,7 +28261,7 @@
         <v>41</v>
       </c>
       <c r="K76" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
@@ -28288,7 +28281,7 @@
         <v>7</v>
       </c>
       <c r="K77" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
@@ -28308,7 +28301,7 @@
         <v>7</v>
       </c>
       <c r="K78" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
@@ -28328,7 +28321,7 @@
         <v>7</v>
       </c>
       <c r="K79" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
@@ -28348,7 +28341,7 @@
         <v>7</v>
       </c>
       <c r="K80" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
@@ -28365,7 +28358,7 @@
         <v>41</v>
       </c>
       <c r="K81" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
@@ -28388,7 +28381,7 @@
         <v>2</v>
       </c>
       <c r="K82" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
@@ -28411,7 +28404,7 @@
         <v>5</v>
       </c>
       <c r="K83" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
@@ -28431,7 +28424,7 @@
         <v>4</v>
       </c>
       <c r="K84" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
@@ -28451,7 +28444,7 @@
         <v>3</v>
       </c>
       <c r="K85" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
@@ -28468,7 +28461,7 @@
         <v>0</v>
       </c>
       <c r="K86" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
@@ -28482,7 +28475,7 @@
         <v>6</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F87" s="1">
         <v>0</v>
@@ -28505,7 +28498,7 @@
         <v>41</v>
       </c>
       <c r="K88" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
@@ -28528,7 +28521,7 @@
         <v>2</v>
       </c>
       <c r="K89" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
@@ -28548,7 +28541,7 @@
         <v>4</v>
       </c>
       <c r="K90" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
@@ -28571,7 +28564,7 @@
         <v>2</v>
       </c>
       <c r="K91" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
@@ -28594,7 +28587,7 @@
         <v>2</v>
       </c>
       <c r="K92" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
@@ -28611,7 +28604,7 @@
         <v>41</v>
       </c>
       <c r="K93" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
@@ -28631,7 +28624,7 @@
         <v>3</v>
       </c>
       <c r="K94" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
@@ -28651,7 +28644,7 @@
         <v>2</v>
       </c>
       <c r="K95" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
@@ -28671,7 +28664,7 @@
         <v>2</v>
       </c>
       <c r="K96" t="s">
-        <v>177</v>
+        <v>248</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
@@ -28685,7 +28678,7 @@
         <v>4</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F97" s="1">
         <v>0</v>
@@ -28708,7 +28701,7 @@
         <v>41</v>
       </c>
       <c r="K98" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
@@ -28728,7 +28721,7 @@
         <v>2</v>
       </c>
       <c r="K99" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
@@ -28748,7 +28741,7 @@
         <v>2</v>
       </c>
       <c r="K100" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.2">
@@ -28768,7 +28761,7 @@
         <v>2</v>
       </c>
       <c r="K101" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.2">
@@ -28788,7 +28781,7 @@
         <v>2</v>
       </c>
       <c r="K102" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
@@ -28805,7 +28798,7 @@
         <v>41</v>
       </c>
       <c r="K103" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
@@ -28825,7 +28818,7 @@
         <v>2</v>
       </c>
       <c r="K104" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
@@ -28867,7 +28860,7 @@
         <v>4</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F107" s="1">
         <v>0</v>
@@ -28890,7 +28883,7 @@
         <v>41</v>
       </c>
       <c r="K108" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
@@ -28963,7 +28956,7 @@
         <v>41</v>
       </c>
       <c r="K113" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.2">
@@ -29000,7 +28993,7 @@
         <v>4</v>
       </c>
       <c r="K115" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.2">
@@ -29020,7 +29013,7 @@
         <v>4</v>
       </c>
       <c r="K116" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.2">
@@ -29040,7 +29033,7 @@
         <v>4</v>
       </c>
       <c r="K117" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.2">
@@ -29060,7 +29053,7 @@
         <v>4</v>
       </c>
       <c r="K118" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.2">
@@ -29080,7 +29073,7 @@
         <v>4</v>
       </c>
       <c r="K119" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.2">
@@ -29100,7 +29093,7 @@
         <v>4</v>
       </c>
       <c r="K120" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.2">
@@ -29120,7 +29113,7 @@
         <v>4</v>
       </c>
       <c r="K121" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.2">
@@ -29134,7 +29127,7 @@
         <v>9</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F122" s="1">
         <v>0</v>
@@ -29157,7 +29150,7 @@
         <v>41</v>
       </c>
       <c r="K123" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.2">
@@ -29177,7 +29170,7 @@
         <v>4</v>
       </c>
       <c r="K124" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.2">
@@ -29197,7 +29190,7 @@
         <v>4</v>
       </c>
       <c r="K125" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.2">
@@ -29217,7 +29210,7 @@
         <v>4</v>
       </c>
       <c r="K126" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.2">
@@ -29237,7 +29230,7 @@
         <v>4</v>
       </c>
       <c r="K127" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.2">
@@ -29254,7 +29247,7 @@
         <v>41</v>
       </c>
       <c r="K128" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.2">
@@ -29327,7 +29320,7 @@
         <v>41</v>
       </c>
       <c r="K133" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.2">
@@ -29400,7 +29393,7 @@
         <v>41</v>
       </c>
       <c r="K138" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.2">
@@ -29456,7 +29449,7 @@
         <v>4</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F142" s="1">
         <v>0</v>
@@ -29479,7 +29472,7 @@
         <v>41</v>
       </c>
       <c r="K143" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.2">
@@ -29552,7 +29545,7 @@
         <v>41</v>
       </c>
       <c r="K148" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.2">
@@ -29569,7 +29562,7 @@
         <v>133</v>
       </c>
       <c r="K149" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.2">
@@ -29592,7 +29585,7 @@
         <v>7</v>
       </c>
       <c r="K150" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.2">
@@ -29615,7 +29608,7 @@
         <v>7</v>
       </c>
       <c r="K151" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.2">
@@ -29638,7 +29631,7 @@
         <v>7</v>
       </c>
       <c r="K152" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.2">
@@ -29661,7 +29654,7 @@
         <v>7</v>
       </c>
       <c r="K153" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.2">
@@ -29684,7 +29677,7 @@
         <v>7</v>
       </c>
       <c r="K154" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.2">
@@ -29707,7 +29700,7 @@
         <v>7</v>
       </c>
       <c r="K155" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.2">
@@ -29730,7 +29723,7 @@
         <v>7</v>
       </c>
       <c r="K156" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.2">
@@ -29753,7 +29746,7 @@
         <v>7</v>
       </c>
       <c r="K157" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.2">
@@ -29776,7 +29769,7 @@
         <v>7</v>
       </c>
       <c r="K158" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.2">
@@ -29799,7 +29792,7 @@
         <v>7</v>
       </c>
       <c r="K159" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.2">
@@ -29813,7 +29806,7 @@
         <v>12</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F160" s="1">
         <v>2</v>
@@ -29825,7 +29818,7 @@
         <v>4</v>
       </c>
       <c r="K160" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.2">
@@ -29842,7 +29835,7 @@
         <v>41</v>
       </c>
       <c r="K161" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.2">
@@ -29865,7 +29858,7 @@
         <v>6</v>
       </c>
       <c r="K162" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.2">
@@ -29888,7 +29881,7 @@
         <v>6</v>
       </c>
       <c r="K163" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.2">
@@ -29911,7 +29904,7 @@
         <v>6</v>
       </c>
       <c r="K164" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.2">
@@ -29934,7 +29927,7 @@
         <v>6</v>
       </c>
       <c r="K165" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.2">
@@ -29951,7 +29944,7 @@
         <v>41</v>
       </c>
       <c r="K166" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.2">
@@ -29974,7 +29967,7 @@
         <v>2</v>
       </c>
       <c r="K167" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.2">
@@ -29997,7 +29990,7 @@
         <v>2</v>
       </c>
       <c r="K168" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.2">
@@ -30020,7 +30013,7 @@
         <v>2</v>
       </c>
       <c r="K169" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.2">
@@ -30043,7 +30036,7 @@
         <v>2</v>
       </c>
       <c r="K170" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.2">
@@ -30066,7 +30059,7 @@
         <v>2</v>
       </c>
       <c r="K171" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.2">
@@ -30089,7 +30082,7 @@
         <v>2</v>
       </c>
       <c r="K172" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.2">
@@ -30112,7 +30105,7 @@
         <v>2</v>
       </c>
       <c r="K173" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.2">
@@ -30135,7 +30128,7 @@
         <v>2</v>
       </c>
       <c r="K174" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.2">
@@ -30149,7 +30142,7 @@
         <v>9</v>
       </c>
       <c r="D175" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F175" s="1">
         <v>0</v>
@@ -30172,7 +30165,7 @@
         <v>41</v>
       </c>
       <c r="K176" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.2">
@@ -30195,7 +30188,7 @@
         <v>2</v>
       </c>
       <c r="K177" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.2">
@@ -30218,7 +30211,7 @@
         <v>2</v>
       </c>
       <c r="K178" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.2">
@@ -30241,7 +30234,7 @@
         <v>2</v>
       </c>
       <c r="K179" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.2">
@@ -30264,7 +30257,7 @@
         <v>2</v>
       </c>
       <c r="K180" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.2">
@@ -30281,7 +30274,7 @@
         <v>41</v>
       </c>
       <c r="K181" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.2">
@@ -30301,7 +30294,7 @@
         <v>3</v>
       </c>
       <c r="K182" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.2">
@@ -30321,7 +30314,7 @@
         <v>3</v>
       </c>
       <c r="K183" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.2">
@@ -30341,7 +30334,7 @@
         <v>3</v>
       </c>
       <c r="K184" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.2">
@@ -30355,13 +30348,13 @@
         <v>4</v>
       </c>
       <c r="D185" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J185" s="1">
         <v>0</v>
       </c>
       <c r="K185" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.2">
@@ -30378,7 +30371,7 @@
         <v>41</v>
       </c>
       <c r="K186" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.2">
@@ -30398,7 +30391,7 @@
         <v>3</v>
       </c>
       <c r="K187" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.2">
@@ -30418,7 +30411,7 @@
         <v>3</v>
       </c>
       <c r="K188" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.2">
@@ -30438,7 +30431,7 @@
         <v>3</v>
       </c>
       <c r="K189" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.2">
@@ -30458,7 +30451,7 @@
         <v>3</v>
       </c>
       <c r="K190" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="191" spans="1:11" x14ac:dyDescent="0.2">
@@ -30475,7 +30468,7 @@
         <v>41</v>
       </c>
       <c r="K191" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="192" spans="1:11" x14ac:dyDescent="0.2">
@@ -30601,7 +30594,7 @@
         <v>9</v>
       </c>
       <c r="D200" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F200" s="1">
         <v>0</v>
@@ -30610,7 +30603,7 @@
         <v>0</v>
       </c>
       <c r="K200" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="201" spans="1:11" x14ac:dyDescent="0.2">
@@ -30627,7 +30620,7 @@
         <v>41</v>
       </c>
       <c r="K201" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="202" spans="1:11" x14ac:dyDescent="0.2">
@@ -30700,7 +30693,7 @@
         <v>41</v>
       </c>
       <c r="K206" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="207" spans="1:11" x14ac:dyDescent="0.2">
@@ -30784,7 +30777,7 @@
         <v>6</v>
       </c>
       <c r="D212" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F212" s="1">
         <v>0</v>
@@ -30807,7 +30800,7 @@
         <v>41</v>
       </c>
       <c r="K213" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.2">
@@ -30880,7 +30873,7 @@
         <v>41</v>
       </c>
       <c r="K218" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="219" spans="1:11" x14ac:dyDescent="0.2">
@@ -30956,7 +30949,7 @@
         <v>2</v>
       </c>
       <c r="K223" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="224" spans="1:11" x14ac:dyDescent="0.2">
@@ -30984,7 +30977,7 @@
         <v>7</v>
       </c>
       <c r="D225" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F225" s="1">
         <v>0</v>
@@ -30993,7 +30986,7 @@
         <v>0</v>
       </c>
       <c r="K225" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="226" spans="1:11" x14ac:dyDescent="0.2">
@@ -31069,7 +31062,7 @@
         <v>1</v>
       </c>
       <c r="K230" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="231" spans="1:11" x14ac:dyDescent="0.2">
@@ -31086,7 +31079,7 @@
         <v>41</v>
       </c>
       <c r="K231" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="232" spans="1:11" x14ac:dyDescent="0.2">
@@ -31142,7 +31135,7 @@
         <v>4</v>
       </c>
       <c r="D235" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F235" s="1">
         <v>0</v>
@@ -31165,7 +31158,7 @@
         <v>41</v>
       </c>
       <c r="K236" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="237" spans="1:11" x14ac:dyDescent="0.2">
@@ -31238,7 +31231,7 @@
         <v>41</v>
       </c>
       <c r="K241" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="242" spans="1:11" x14ac:dyDescent="0.2">
@@ -31272,7 +31265,7 @@
         <v>4</v>
       </c>
       <c r="K243" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.2">
@@ -31292,7 +31285,7 @@
         <v>8</v>
       </c>
       <c r="K244" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.2">
@@ -31312,7 +31305,7 @@
         <v>8</v>
       </c>
       <c r="K245" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="246" spans="1:11" x14ac:dyDescent="0.2">
@@ -31332,7 +31325,7 @@
         <v>4</v>
       </c>
       <c r="K246" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="247" spans="1:11" x14ac:dyDescent="0.2">
@@ -31346,7 +31339,7 @@
         <v>6</v>
       </c>
       <c r="D247" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F247" s="1">
         <v>0</v>
@@ -31369,7 +31362,7 @@
         <v>41</v>
       </c>
       <c r="K248" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="249" spans="1:11" x14ac:dyDescent="0.2">
@@ -31389,7 +31382,7 @@
         <v>4</v>
       </c>
       <c r="K249" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.2">
@@ -31423,7 +31416,7 @@
         <v>4</v>
       </c>
       <c r="K251" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="252" spans="1:11" x14ac:dyDescent="0.2">
@@ -31443,7 +31436,7 @@
         <v>4</v>
       </c>
       <c r="K252" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="253" spans="1:11" x14ac:dyDescent="0.2">
@@ -31460,7 +31453,7 @@
         <v>41</v>
       </c>
       <c r="K253" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="254" spans="1:11" x14ac:dyDescent="0.2">
@@ -31480,7 +31473,7 @@
         <v>2</v>
       </c>
       <c r="K254" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="255" spans="1:11" x14ac:dyDescent="0.2">
@@ -31500,7 +31493,7 @@
         <v>2</v>
       </c>
       <c r="K255" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.2">
@@ -31520,7 +31513,7 @@
         <v>2</v>
       </c>
       <c r="K256" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="257" spans="1:11" x14ac:dyDescent="0.2">
@@ -31540,7 +31533,7 @@
         <v>2</v>
       </c>
       <c r="K257" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="258" spans="1:11" x14ac:dyDescent="0.2">
@@ -31560,7 +31553,7 @@
         <v>2</v>
       </c>
       <c r="K258" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="259" spans="1:11" x14ac:dyDescent="0.2">
@@ -31580,7 +31573,7 @@
         <v>2</v>
       </c>
       <c r="K259" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="260" spans="1:11" x14ac:dyDescent="0.2">
@@ -31600,7 +31593,7 @@
         <v>2</v>
       </c>
       <c r="K260" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="261" spans="1:11" x14ac:dyDescent="0.2">
@@ -31620,7 +31613,7 @@
         <v>2</v>
       </c>
       <c r="K261" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="262" spans="1:11" x14ac:dyDescent="0.2">
@@ -31634,7 +31627,7 @@
         <v>9</v>
       </c>
       <c r="D262" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F262" s="1">
         <v>2</v>
@@ -31646,7 +31639,7 @@
         <v>10</v>
       </c>
       <c r="K262" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="263" spans="1:11" x14ac:dyDescent="0.2">
@@ -31663,7 +31656,7 @@
         <v>41</v>
       </c>
       <c r="K263" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="264" spans="1:11" x14ac:dyDescent="0.2">
@@ -31683,7 +31676,7 @@
         <v>2</v>
       </c>
       <c r="K264" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="265" spans="1:11" x14ac:dyDescent="0.2">
@@ -31703,7 +31696,7 @@
         <v>2</v>
       </c>
       <c r="K265" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="266" spans="1:11" x14ac:dyDescent="0.2">
@@ -31723,7 +31716,7 @@
         <v>2</v>
       </c>
       <c r="K266" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="267" spans="1:11" x14ac:dyDescent="0.2">
@@ -31743,7 +31736,7 @@
         <v>2</v>
       </c>
       <c r="K267" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="268" spans="1:11" x14ac:dyDescent="0.2">
@@ -31760,7 +31753,7 @@
         <v>41</v>
       </c>
       <c r="K268" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="269" spans="1:11" x14ac:dyDescent="0.2">
@@ -31780,7 +31773,7 @@
         <v>3</v>
       </c>
       <c r="K269" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="270" spans="1:11" x14ac:dyDescent="0.2">
@@ -31800,7 +31793,7 @@
         <v>1</v>
       </c>
       <c r="K270" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="271" spans="1:11" x14ac:dyDescent="0.2">
@@ -31820,7 +31813,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="272" spans="1:11" x14ac:dyDescent="0.2">
@@ -31834,7 +31827,7 @@
         <v>4</v>
       </c>
       <c r="D272" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F272" s="1">
         <v>1</v>
@@ -31846,7 +31839,7 @@
         <v>11</v>
       </c>
       <c r="K272" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.2">
@@ -31866,7 +31859,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="274" spans="1:11" x14ac:dyDescent="0.2">
@@ -31939,7 +31932,7 @@
         <v>41</v>
       </c>
       <c r="K278" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="279" spans="1:11" x14ac:dyDescent="0.2">
@@ -31995,7 +31988,7 @@
         <v>4</v>
       </c>
       <c r="D282" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F282" s="1">
         <v>0</v>
@@ -32018,7 +32011,7 @@
         <v>41</v>
       </c>
       <c r="K283" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="284" spans="1:11" x14ac:dyDescent="0.2">
@@ -32077,7 +32070,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="288" spans="1:11" x14ac:dyDescent="0.2">
@@ -32094,7 +32087,7 @@
         <v>41</v>
       </c>
       <c r="K288" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="289" spans="1:11" x14ac:dyDescent="0.2">
@@ -32114,7 +32107,7 @@
         <v>8</v>
       </c>
       <c r="K289" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="290" spans="1:11" x14ac:dyDescent="0.2">
@@ -32134,7 +32127,7 @@
         <v>8</v>
       </c>
       <c r="K290" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="291" spans="1:11" x14ac:dyDescent="0.2">
@@ -32154,7 +32147,7 @@
         <v>8</v>
       </c>
       <c r="K291" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="292" spans="1:11" x14ac:dyDescent="0.2">
@@ -32168,7 +32161,7 @@
         <v>4</v>
       </c>
       <c r="D292" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F292" s="1">
         <v>8</v>
@@ -32180,7 +32173,7 @@
         <v>15</v>
       </c>
       <c r="K292" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="293" spans="1:11" x14ac:dyDescent="0.2">
@@ -32197,7 +32190,7 @@
         <v>41</v>
       </c>
       <c r="K293" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="294" spans="1:11" x14ac:dyDescent="0.2">
@@ -32217,7 +32210,7 @@
         <v>8</v>
       </c>
       <c r="K294" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="295" spans="1:11" x14ac:dyDescent="0.2">
@@ -32237,7 +32230,7 @@
         <v>7</v>
       </c>
       <c r="K295" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="296" spans="1:11" x14ac:dyDescent="0.2">
@@ -32257,7 +32250,7 @@
         <v>7</v>
       </c>
       <c r="K296" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="297" spans="1:11" x14ac:dyDescent="0.2">
@@ -32277,7 +32270,7 @@
         <v>7</v>
       </c>
       <c r="K297" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="298" spans="1:11" x14ac:dyDescent="0.2">
@@ -32294,7 +32287,7 @@
         <v>41</v>
       </c>
       <c r="K298" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="299" spans="1:11" x14ac:dyDescent="0.2">
@@ -32320,7 +32313,7 @@
         <v>2</v>
       </c>
       <c r="K299" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="300" spans="1:11" x14ac:dyDescent="0.2">
@@ -32340,7 +32333,7 @@
         <v>2</v>
       </c>
       <c r="K300" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="301" spans="1:11" x14ac:dyDescent="0.2">
@@ -32360,7 +32353,7 @@
         <v>4</v>
       </c>
       <c r="K301" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="302" spans="1:11" x14ac:dyDescent="0.2">
@@ -32380,7 +32373,7 @@
         <v>2</v>
       </c>
       <c r="K302" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="303" spans="1:11" x14ac:dyDescent="0.2">
@@ -32400,7 +32393,7 @@
         <v>2</v>
       </c>
       <c r="K303" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="304" spans="1:11" x14ac:dyDescent="0.2">
@@ -32414,7 +32407,7 @@
         <v>6</v>
       </c>
       <c r="D304" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F304" s="1">
         <v>0</v>
@@ -32437,7 +32430,7 @@
         <v>41</v>
       </c>
       <c r="K305" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="306" spans="1:11" x14ac:dyDescent="0.2">
@@ -32457,7 +32450,7 @@
         <v>2</v>
       </c>
       <c r="K306" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="307" spans="1:11" x14ac:dyDescent="0.2">
@@ -32477,7 +32470,7 @@
         <v>2</v>
       </c>
       <c r="K307" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="308" spans="1:11" x14ac:dyDescent="0.2">
@@ -32497,7 +32490,7 @@
         <v>2</v>
       </c>
       <c r="K308" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="309" spans="1:11" x14ac:dyDescent="0.2">
@@ -32517,7 +32510,7 @@
         <v>2</v>
       </c>
       <c r="K309" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="310" spans="1:11" x14ac:dyDescent="0.2">
@@ -32534,7 +32527,7 @@
         <v>41</v>
       </c>
       <c r="K310" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="311" spans="1:11" x14ac:dyDescent="0.2">
@@ -32578,7 +32571,7 @@
         <v>3</v>
       </c>
       <c r="D313" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F313" s="1">
         <v>0</v>
@@ -32587,7 +32580,7 @@
         <v>8</v>
       </c>
       <c r="K313" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="314" spans="1:11" x14ac:dyDescent="0.2">
@@ -32634,7 +32627,7 @@
         <v>41</v>
       </c>
       <c r="K316" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="317" spans="1:11" x14ac:dyDescent="0.2">
@@ -32670,7 +32663,7 @@
         <v>1</v>
       </c>
       <c r="K318" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="319" spans="1:11" x14ac:dyDescent="0.2">
@@ -32691,7 +32684,7 @@
         <v>1</v>
       </c>
       <c r="K319" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="320" spans="1:11" x14ac:dyDescent="0.2">
@@ -32712,7 +32705,7 @@
         <v>1</v>
       </c>
       <c r="K320" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="321" spans="1:11" x14ac:dyDescent="0.2">
@@ -32729,7 +32722,7 @@
         <v>41</v>
       </c>
       <c r="K321" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="322" spans="1:11" x14ac:dyDescent="0.2">
@@ -32743,7 +32736,7 @@
         <v>1</v>
       </c>
       <c r="D322" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F322" s="1">
         <v>0</v>
@@ -32752,7 +32745,7 @@
         <v>13</v>
       </c>
       <c r="K322" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="323" spans="1:11" x14ac:dyDescent="0.2">
@@ -32773,7 +32766,7 @@
         <v>3</v>
       </c>
       <c r="K323" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="324" spans="1:11" x14ac:dyDescent="0.2">
@@ -32794,7 +32787,7 @@
         <v>3</v>
       </c>
       <c r="K324" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="325" spans="1:11" x14ac:dyDescent="0.2">
@@ -32815,7 +32808,7 @@
         <v>3</v>
       </c>
       <c r="K325" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="326" spans="1:11" x14ac:dyDescent="0.2">
@@ -32829,7 +32822,7 @@
         <v>5</v>
       </c>
       <c r="D326" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F326" s="1">
         <v>0</v>
@@ -32852,7 +32845,7 @@
         <v>41</v>
       </c>
       <c r="K327" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="328" spans="1:11" x14ac:dyDescent="0.2">
@@ -32873,7 +32866,7 @@
         <v>3</v>
       </c>
       <c r="K328" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="329" spans="1:11" x14ac:dyDescent="0.2">
@@ -32894,7 +32887,7 @@
         <v>3</v>
       </c>
       <c r="K329" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="330" spans="1:11" x14ac:dyDescent="0.2">
@@ -32918,7 +32911,7 @@
         <v>3</v>
       </c>
       <c r="K330" t="s">
-        <v>210</v>
+        <v>245</v>
       </c>
     </row>
     <row r="331" spans="1:11" x14ac:dyDescent="0.2">
@@ -32939,7 +32932,7 @@
         <v>3</v>
       </c>
       <c r="K331" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="332" spans="1:11" x14ac:dyDescent="0.2">
@@ -32956,7 +32949,7 @@
         <v>41</v>
       </c>
       <c r="K332" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="333" spans="1:11" x14ac:dyDescent="0.2">
@@ -32977,7 +32970,7 @@
         <v>5</v>
       </c>
       <c r="K333" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="334" spans="1:11" x14ac:dyDescent="0.2">
@@ -32998,7 +32991,7 @@
         <v>5</v>
       </c>
       <c r="K334" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="335" spans="1:11" x14ac:dyDescent="0.2">
@@ -33019,7 +33012,7 @@
         <v>5</v>
       </c>
       <c r="K335" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="336" spans="1:11" x14ac:dyDescent="0.2">
@@ -33040,7 +33033,7 @@
         <v>5</v>
       </c>
       <c r="K336" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="337" spans="1:11" x14ac:dyDescent="0.2">
@@ -33061,7 +33054,7 @@
         <v>5</v>
       </c>
       <c r="K337" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="338" spans="1:11" x14ac:dyDescent="0.2">
@@ -33082,7 +33075,7 @@
         <v>5</v>
       </c>
       <c r="K338" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="339" spans="1:11" x14ac:dyDescent="0.2">
@@ -33117,7 +33110,7 @@
         <v>5</v>
       </c>
       <c r="K340" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="341" spans="1:11" x14ac:dyDescent="0.2">
@@ -33138,7 +33131,7 @@
         <v>5</v>
       </c>
       <c r="K341" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="342" spans="1:11" x14ac:dyDescent="0.2">
@@ -33159,7 +33152,7 @@
         <v>5</v>
       </c>
       <c r="K342" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="343" spans="1:11" x14ac:dyDescent="0.2">
@@ -33173,7 +33166,7 @@
         <v>11</v>
       </c>
       <c r="D343" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F343" s="1">
         <v>5</v>
@@ -33185,7 +33178,7 @@
         <v>13</v>
       </c>
       <c r="K343" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="344" spans="1:11" x14ac:dyDescent="0.2">
@@ -33202,7 +33195,7 @@
         <v>41</v>
       </c>
       <c r="K344" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="345" spans="1:11" x14ac:dyDescent="0.2">
@@ -33279,7 +33272,7 @@
         <v>41</v>
       </c>
       <c r="K349" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="350" spans="1:11" x14ac:dyDescent="0.2">
@@ -33338,7 +33331,7 @@
         <v>4</v>
       </c>
       <c r="D353" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F353" s="1">
         <v>0</v>
@@ -33347,7 +33340,7 @@
         <v>13</v>
       </c>
       <c r="K353" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="354" spans="1:11" x14ac:dyDescent="0.2">
@@ -33364,7 +33357,7 @@
         <v>41</v>
       </c>
       <c r="K354" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="355" spans="1:11" x14ac:dyDescent="0.2">
@@ -33441,7 +33434,7 @@
         <v>41</v>
       </c>
       <c r="K359" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="360" spans="1:11" x14ac:dyDescent="0.2">
@@ -33500,7 +33493,7 @@
         <v>4</v>
       </c>
       <c r="D363" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G363" s="1">
         <v>0</v>
@@ -33523,7 +33516,7 @@
         <v>41</v>
       </c>
       <c r="K364" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="365" spans="1:11" x14ac:dyDescent="0.2">
@@ -33544,7 +33537,7 @@
         <v>2</v>
       </c>
       <c r="K365" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="366" spans="1:11" x14ac:dyDescent="0.2">
@@ -33565,7 +33558,7 @@
         <v>2</v>
       </c>
       <c r="K366" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="367" spans="1:11" x14ac:dyDescent="0.2">
@@ -33586,7 +33579,7 @@
         <v>2</v>
       </c>
       <c r="K367" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="368" spans="1:11" x14ac:dyDescent="0.2">
@@ -33607,7 +33600,7 @@
         <v>2</v>
       </c>
       <c r="K368" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="369" spans="1:11" x14ac:dyDescent="0.2">
@@ -33624,7 +33617,7 @@
         <v>41</v>
       </c>
       <c r="K369" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="370" spans="1:11" x14ac:dyDescent="0.2">
@@ -33645,7 +33638,7 @@
         <v>2</v>
       </c>
       <c r="K370" t="s">
-        <v>215</v>
+        <v>246</v>
       </c>
     </row>
     <row r="371" spans="1:11" x14ac:dyDescent="0.2">
@@ -33719,7 +33712,7 @@
         <v>6</v>
       </c>
       <c r="D375" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F375" s="1">
         <v>0</v>
@@ -33742,7 +33735,7 @@
         <v>41</v>
       </c>
       <c r="K376" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="377" spans="1:11" x14ac:dyDescent="0.2">
@@ -33819,7 +33812,7 @@
         <v>41</v>
       </c>
       <c r="K381" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="382" spans="1:11" x14ac:dyDescent="0.2">
@@ -33840,7 +33833,7 @@
         <v>9</v>
       </c>
       <c r="K382" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="383" spans="1:11" x14ac:dyDescent="0.2">
@@ -33864,7 +33857,7 @@
         <v>7</v>
       </c>
       <c r="K383" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="384" spans="1:11" x14ac:dyDescent="0.2">
@@ -33885,7 +33878,7 @@
         <v>9</v>
       </c>
       <c r="K384" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="385" spans="1:11" x14ac:dyDescent="0.2">
@@ -33909,7 +33902,7 @@
         <v>7</v>
       </c>
       <c r="K385" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="386" spans="1:11" x14ac:dyDescent="0.2">
@@ -33930,7 +33923,7 @@
         <v>9</v>
       </c>
       <c r="K386" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="387" spans="1:11" x14ac:dyDescent="0.2">
@@ -33951,7 +33944,7 @@
         <v>9</v>
       </c>
       <c r="K387" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="388" spans="1:11" x14ac:dyDescent="0.2">
@@ -33972,7 +33965,7 @@
         <v>9</v>
       </c>
       <c r="K388" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="389" spans="1:11" x14ac:dyDescent="0.2">
@@ -33993,7 +33986,7 @@
         <v>9</v>
       </c>
       <c r="K389" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="390" spans="1:11" x14ac:dyDescent="0.2">
@@ -34007,7 +34000,7 @@
         <v>9</v>
       </c>
       <c r="D390" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F390" s="1">
         <v>3</v>
@@ -34019,7 +34012,7 @@
         <v>4</v>
       </c>
       <c r="K390" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="391" spans="1:11" x14ac:dyDescent="0.2">
@@ -34054,7 +34047,7 @@
         <v>9</v>
       </c>
       <c r="K392" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="393" spans="1:11" x14ac:dyDescent="0.2">
@@ -34075,7 +34068,7 @@
         <v>9</v>
       </c>
       <c r="K393" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="394" spans="1:11" x14ac:dyDescent="0.2">
@@ -34096,7 +34089,7 @@
         <v>9</v>
       </c>
       <c r="K394" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="395" spans="1:11" x14ac:dyDescent="0.2">
@@ -34117,7 +34110,7 @@
         <v>9</v>
       </c>
       <c r="K395" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="396" spans="1:11" x14ac:dyDescent="0.2">
@@ -34134,7 +34127,7 @@
         <v>41</v>
       </c>
       <c r="K396" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="397" spans="1:11" x14ac:dyDescent="0.2">
@@ -34155,7 +34148,7 @@
         <v>1</v>
       </c>
       <c r="K397" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="398" spans="1:11" x14ac:dyDescent="0.2">
@@ -34218,7 +34211,7 @@
         <v>0</v>
       </c>
       <c r="K401" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="402" spans="1:11" x14ac:dyDescent="0.2">
@@ -34235,7 +34228,7 @@
         <v>41</v>
       </c>
       <c r="K402" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="403" spans="1:11" x14ac:dyDescent="0.2">
@@ -34312,7 +34305,7 @@
         <v>41</v>
       </c>
       <c r="K407" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="408" spans="1:11" x14ac:dyDescent="0.2">
@@ -34333,7 +34326,7 @@
         <v>3</v>
       </c>
       <c r="K408" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="409" spans="1:11" x14ac:dyDescent="0.2">
@@ -34354,7 +34347,7 @@
         <v>3</v>
       </c>
       <c r="K409" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="410" spans="1:11" x14ac:dyDescent="0.2">
@@ -34368,7 +34361,7 @@
         <v>3</v>
       </c>
       <c r="D410" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F410" s="1">
         <v>0</v>
@@ -34409,7 +34402,7 @@
         <v>3</v>
       </c>
       <c r="K412" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="413" spans="1:11" x14ac:dyDescent="0.2">
@@ -34430,7 +34423,7 @@
         <v>3</v>
       </c>
       <c r="K413" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="414" spans="1:11" x14ac:dyDescent="0.2">
@@ -34451,7 +34444,7 @@
         <v>3</v>
       </c>
       <c r="K414" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="415" spans="1:11" x14ac:dyDescent="0.2">
@@ -34472,7 +34465,7 @@
         <v>3</v>
       </c>
       <c r="K415" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="416" spans="1:11" x14ac:dyDescent="0.2">
@@ -34489,7 +34482,7 @@
         <v>41</v>
       </c>
       <c r="K416" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="417" spans="1:11" x14ac:dyDescent="0.2">
@@ -34610,7 +34603,7 @@
         <v>8</v>
       </c>
       <c r="D424" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F424" s="1">
         <v>0</v>
@@ -34619,7 +34612,7 @@
         <v>9</v>
       </c>
       <c r="K424" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="425" spans="1:11" x14ac:dyDescent="0.2">
@@ -34636,7 +34629,7 @@
         <v>41</v>
       </c>
       <c r="K425" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="426" spans="1:11" x14ac:dyDescent="0.2">
@@ -34713,7 +34706,7 @@
         <v>41</v>
       </c>
       <c r="K430" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="431" spans="1:11" x14ac:dyDescent="0.2">
@@ -34787,13 +34780,13 @@
         <v>5</v>
       </c>
       <c r="D435" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J435" s="1">
         <v>12</v>
       </c>
       <c r="K435" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="436" spans="1:11" x14ac:dyDescent="0.2">
@@ -34810,7 +34803,7 @@
         <v>41</v>
       </c>
       <c r="K436" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="437" spans="1:11" x14ac:dyDescent="0.2">
@@ -34887,7 +34880,7 @@
         <v>41</v>
       </c>
       <c r="K441" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="442" spans="1:11" x14ac:dyDescent="0.2">
@@ -34904,7 +34897,7 @@
         <v>133</v>
       </c>
       <c r="K442" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="443" spans="1:11" x14ac:dyDescent="0.2">
@@ -34963,7 +34956,7 @@
         <v>5</v>
       </c>
       <c r="D446" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F446" s="1">
         <v>0</v>
@@ -34986,7 +34979,7 @@
         <v>41</v>
       </c>
       <c r="K447" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="448" spans="1:11" x14ac:dyDescent="0.2">
@@ -35063,7 +35056,7 @@
         <v>41</v>
       </c>
       <c r="K452" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="453" spans="1:11" x14ac:dyDescent="0.2">
@@ -35087,7 +35080,7 @@
         <v>2</v>
       </c>
       <c r="K453" t="s">
-        <v>222</v>
+        <v>247</v>
       </c>
     </row>
     <row r="454" spans="1:11" x14ac:dyDescent="0.2">
@@ -35120,7 +35113,7 @@
         <v>0</v>
       </c>
       <c r="K455" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="456" spans="1:11" x14ac:dyDescent="0.2">
@@ -35179,7 +35172,7 @@
         <v>7</v>
       </c>
       <c r="D459" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F459" s="1">
         <v>0</v>
@@ -35276,7 +35269,7 @@
         <v>41</v>
       </c>
       <c r="K465" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="466" spans="1:11" x14ac:dyDescent="0.2">
@@ -35395,7 +35388,7 @@
         <v>8</v>
       </c>
       <c r="D473" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F473" s="1">
         <v>0</v>
@@ -35404,7 +35397,7 @@
         <v>11</v>
       </c>
       <c r="K473" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="474" spans="1:11" x14ac:dyDescent="0.2">
@@ -35421,7 +35414,7 @@
         <v>41</v>
       </c>
       <c r="K474" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="475" spans="1:11" x14ac:dyDescent="0.2">
@@ -35498,7 +35491,7 @@
         <v>41</v>
       </c>
       <c r="K479" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="480" spans="1:11" x14ac:dyDescent="0.2">
@@ -35576,7 +35569,7 @@
         <v>0</v>
       </c>
       <c r="K484" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
     <row r="485" spans="1:11" x14ac:dyDescent="0.2">
@@ -35593,7 +35586,7 @@
         <v>41</v>
       </c>
       <c r="K485" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="486" spans="1:11" x14ac:dyDescent="0.2">
@@ -35670,7 +35663,7 @@
         <v>41</v>
       </c>
       <c r="K490" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="491" spans="1:11" x14ac:dyDescent="0.2">
@@ -35691,7 +35684,7 @@
         <v>3</v>
       </c>
       <c r="K491" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
     </row>
     <row r="492" spans="1:11" x14ac:dyDescent="0.2">
@@ -35712,7 +35705,7 @@
         <v>3</v>
       </c>
       <c r="K492" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
     </row>
     <row r="493" spans="1:11" x14ac:dyDescent="0.2">
@@ -35733,7 +35726,7 @@
         <v>3</v>
       </c>
       <c r="K493" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
     </row>
     <row r="494" spans="1:11" x14ac:dyDescent="0.2">
@@ -35747,7 +35740,7 @@
         <v>4</v>
       </c>
       <c r="D494" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F494" s="1">
         <v>0</v>
@@ -35756,7 +35749,7 @@
         <v>2</v>
       </c>
       <c r="K494" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="495" spans="1:11" x14ac:dyDescent="0.2">
@@ -35773,7 +35766,7 @@
         <v>41</v>
       </c>
       <c r="K495" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="496" spans="1:11" x14ac:dyDescent="0.2">
@@ -35794,7 +35787,7 @@
         <v>2</v>
       </c>
       <c r="K496" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="497" spans="1:11" x14ac:dyDescent="0.2">
@@ -35815,7 +35808,7 @@
         <v>2</v>
       </c>
       <c r="K497" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="498" spans="1:11" x14ac:dyDescent="0.2">
@@ -35836,7 +35829,7 @@
         <v>2</v>
       </c>
       <c r="K498" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="499" spans="1:11" x14ac:dyDescent="0.2">
@@ -35857,7 +35850,7 @@
         <v>2</v>
       </c>
       <c r="K499" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="500" spans="1:11" x14ac:dyDescent="0.2">
@@ -35874,7 +35867,7 @@
         <v>41</v>
       </c>
       <c r="K500" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="501" spans="1:11" x14ac:dyDescent="0.2">
@@ -35895,7 +35888,7 @@
         <v>4</v>
       </c>
       <c r="K501" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="502" spans="1:11" x14ac:dyDescent="0.2">
@@ -35916,7 +35909,7 @@
         <v>4</v>
       </c>
       <c r="K502" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="503" spans="1:11" x14ac:dyDescent="0.2">
@@ -35937,7 +35930,7 @@
         <v>4</v>
       </c>
       <c r="K503" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="504" spans="1:11" x14ac:dyDescent="0.2">
@@ -35958,7 +35951,7 @@
         <v>4</v>
       </c>
       <c r="K504" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="505" spans="1:11" x14ac:dyDescent="0.2">
@@ -35979,7 +35972,7 @@
         <v>4</v>
       </c>
       <c r="K505" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="506" spans="1:11" x14ac:dyDescent="0.2">
@@ -35993,7 +35986,7 @@
         <v>6</v>
       </c>
       <c r="D506" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F506" s="1">
         <v>2</v>
@@ -36005,7 +35998,7 @@
         <v>8</v>
       </c>
       <c r="K506" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
     </row>
     <row r="507" spans="1:11" x14ac:dyDescent="0.2">
@@ -36022,7 +36015,7 @@
         <v>41</v>
       </c>
       <c r="K507" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="508" spans="1:11" x14ac:dyDescent="0.2">
@@ -36043,7 +36036,7 @@
         <v>4</v>
       </c>
       <c r="K508" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="509" spans="1:11" x14ac:dyDescent="0.2">
@@ -36064,7 +36057,7 @@
         <v>4</v>
       </c>
       <c r="K509" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="510" spans="1:11" x14ac:dyDescent="0.2">
@@ -36085,7 +36078,7 @@
         <v>4</v>
       </c>
       <c r="K510" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="511" spans="1:11" x14ac:dyDescent="0.2">
@@ -36106,7 +36099,7 @@
         <v>4</v>
       </c>
       <c r="K511" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="512" spans="1:11" x14ac:dyDescent="0.2">
@@ -36123,7 +36116,7 @@
         <v>41</v>
       </c>
       <c r="K512" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="513" spans="1:11" x14ac:dyDescent="0.2">
@@ -36161,7 +36154,7 @@
         <v>7</v>
       </c>
       <c r="K514" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="515" spans="1:11" x14ac:dyDescent="0.2">
@@ -36199,7 +36192,7 @@
         <v>7</v>
       </c>
       <c r="K516" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="517" spans="1:11" x14ac:dyDescent="0.2">
@@ -36220,7 +36213,7 @@
         <v>7</v>
       </c>
       <c r="K517" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="518" spans="1:11" x14ac:dyDescent="0.2">
@@ -36241,7 +36234,7 @@
         <v>7</v>
       </c>
       <c r="K518" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="519" spans="1:11" x14ac:dyDescent="0.2">
@@ -36262,7 +36255,7 @@
         <v>7</v>
       </c>
       <c r="K519" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="520" spans="1:11" x14ac:dyDescent="0.2">
@@ -36283,7 +36276,7 @@
         <v>7</v>
       </c>
       <c r="K520" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="521" spans="1:11" x14ac:dyDescent="0.2">
@@ -36297,7 +36290,7 @@
         <v>9</v>
       </c>
       <c r="D521" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F521" s="1">
         <v>5</v>
@@ -36309,7 +36302,7 @@
         <v>8</v>
       </c>
       <c r="K521" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
     </row>
     <row r="522" spans="1:11" x14ac:dyDescent="0.2">
@@ -36326,7 +36319,7 @@
         <v>41</v>
       </c>
       <c r="K522" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
     </row>
     <row r="523" spans="1:11" x14ac:dyDescent="0.2">
@@ -36347,7 +36340,7 @@
         <v>7</v>
       </c>
       <c r="K523" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="524" spans="1:11" x14ac:dyDescent="0.2">
@@ -36368,7 +36361,7 @@
         <v>7</v>
       </c>
       <c r="K524" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="525" spans="1:11" x14ac:dyDescent="0.2">
@@ -36389,7 +36382,7 @@
         <v>7</v>
       </c>
       <c r="K525" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="526" spans="1:11" x14ac:dyDescent="0.2">
@@ -36410,7 +36403,7 @@
         <v>7</v>
       </c>
       <c r="K526" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
     </row>
     <row r="527" spans="1:11" x14ac:dyDescent="0.2">
@@ -36427,7 +36420,7 @@
         <v>41</v>
       </c>
       <c r="K527" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="528" spans="1:11" x14ac:dyDescent="0.2">
@@ -36448,7 +36441,7 @@
         <v>4</v>
       </c>
       <c r="K528" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="529" spans="1:11" x14ac:dyDescent="0.2">
@@ -36469,7 +36462,7 @@
         <v>4</v>
       </c>
       <c r="K529" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="530" spans="1:11" x14ac:dyDescent="0.2">
@@ -36507,7 +36500,7 @@
         <v>4</v>
       </c>
       <c r="K531" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="532" spans="1:11" x14ac:dyDescent="0.2">
@@ -36528,7 +36521,7 @@
         <v>4</v>
       </c>
       <c r="K532" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="533" spans="1:11" x14ac:dyDescent="0.2">
@@ -36545,7 +36538,7 @@
         <v>41</v>
       </c>
       <c r="K533" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="534" spans="1:11" x14ac:dyDescent="0.2">
@@ -36566,7 +36559,7 @@
         <v>4</v>
       </c>
       <c r="K534" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="535" spans="1:11" x14ac:dyDescent="0.2">
@@ -36587,7 +36580,7 @@
         <v>4</v>
       </c>
       <c r="K535" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="536" spans="1:11" x14ac:dyDescent="0.2">
@@ -36608,7 +36601,7 @@
         <v>4</v>
       </c>
       <c r="K536" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="537" spans="1:11" x14ac:dyDescent="0.2">
@@ -36629,7 +36622,7 @@
         <v>4</v>
       </c>
       <c r="K537" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="538" spans="1:11" x14ac:dyDescent="0.2">
@@ -36646,7 +36639,7 @@
         <v>41</v>
       </c>
       <c r="K538" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="539" spans="1:11" x14ac:dyDescent="0.2">
@@ -36724,7 +36717,7 @@
         <v>0</v>
       </c>
       <c r="K543" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
     </row>
     <row r="544" spans="1:11" x14ac:dyDescent="0.2">
@@ -36815,7 +36808,7 @@
         <v>41</v>
       </c>
       <c r="K549" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="550" spans="1:11" x14ac:dyDescent="0.2">
@@ -36836,7 +36829,7 @@
         <v>2</v>
       </c>
       <c r="K550" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="551" spans="1:11" x14ac:dyDescent="0.2">
@@ -36857,7 +36850,7 @@
         <v>2</v>
       </c>
       <c r="K551" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="552" spans="1:11" x14ac:dyDescent="0.2">
@@ -36878,7 +36871,7 @@
         <v>2</v>
       </c>
       <c r="K552" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="553" spans="1:11" x14ac:dyDescent="0.2">
@@ -36899,7 +36892,7 @@
         <v>2</v>
       </c>
       <c r="K553" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="554" spans="1:11" x14ac:dyDescent="0.2">
@@ -36920,7 +36913,7 @@
         <v>2</v>
       </c>
       <c r="K554" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="555" spans="1:11" x14ac:dyDescent="0.2">
@@ -36941,7 +36934,7 @@
         <v>2</v>
       </c>
       <c r="K555" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="556" spans="1:11" x14ac:dyDescent="0.2">
@@ -36962,7 +36955,7 @@
         <v>2</v>
       </c>
       <c r="K556" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="557" spans="1:11" x14ac:dyDescent="0.2">
@@ -36983,7 +36976,7 @@
         <v>2</v>
       </c>
       <c r="K557" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="558" spans="1:11" x14ac:dyDescent="0.2">
@@ -37004,7 +36997,7 @@
         <v>2</v>
       </c>
       <c r="K558" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="559" spans="1:11" x14ac:dyDescent="0.2">
@@ -37025,7 +37018,7 @@
         <v>2</v>
       </c>
       <c r="K559" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="560" spans="1:11" x14ac:dyDescent="0.2">
@@ -37046,7 +37039,7 @@
         <v>2</v>
       </c>
       <c r="K560" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="561" spans="1:11" x14ac:dyDescent="0.2">
@@ -37060,7 +37053,7 @@
         <v>12</v>
       </c>
       <c r="D561" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F561" s="1">
         <v>2</v>
@@ -37072,7 +37065,7 @@
         <v>13</v>
       </c>
       <c r="K561" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="562" spans="1:11" x14ac:dyDescent="0.2">
@@ -37107,7 +37100,7 @@
         <v>2</v>
       </c>
       <c r="K563" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="564" spans="1:11" x14ac:dyDescent="0.2">
@@ -37128,7 +37121,7 @@
         <v>2</v>
       </c>
       <c r="K564" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="565" spans="1:11" x14ac:dyDescent="0.2">
@@ -37149,7 +37142,7 @@
         <v>2</v>
       </c>
       <c r="K565" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="566" spans="1:11" x14ac:dyDescent="0.2">
@@ -37170,7 +37163,7 @@
         <v>2</v>
       </c>
       <c r="K566" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="567" spans="1:11" x14ac:dyDescent="0.2">
@@ -37187,7 +37180,7 @@
         <v>41</v>
       </c>
       <c r="K567" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="568" spans="1:11" x14ac:dyDescent="0.2">
@@ -37276,7 +37269,7 @@
         <v>6</v>
       </c>
       <c r="D573" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F573" s="1">
         <v>0</v>
@@ -37299,7 +37292,7 @@
         <v>41</v>
       </c>
       <c r="K574" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="575" spans="1:11" x14ac:dyDescent="0.2">
@@ -37376,7 +37369,7 @@
         <v>41</v>
       </c>
       <c r="K579" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="580" spans="1:11" x14ac:dyDescent="0.2">
@@ -37403,7 +37396,7 @@
         <v>1</v>
       </c>
       <c r="K580" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
     </row>
     <row r="581" spans="1:11" x14ac:dyDescent="0.2">
@@ -37427,7 +37420,7 @@
         <v>1</v>
       </c>
       <c r="K581" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
     </row>
     <row r="582" spans="1:11" x14ac:dyDescent="0.2">
@@ -37451,7 +37444,7 @@
         <v>1</v>
       </c>
       <c r="K582" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
     </row>
     <row r="583" spans="1:11" x14ac:dyDescent="0.2">
@@ -37475,7 +37468,7 @@
         <v>2</v>
       </c>
       <c r="K583" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
     </row>
     <row r="584" spans="1:11" x14ac:dyDescent="0.2">
@@ -37489,7 +37482,7 @@
         <v>5</v>
       </c>
       <c r="D584" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F584" s="1">
         <v>0</v>
@@ -37533,7 +37526,7 @@
         <v>2</v>
       </c>
       <c r="K586" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
     </row>
     <row r="587" spans="1:11" x14ac:dyDescent="0.2">
@@ -37554,7 +37547,7 @@
         <v>1</v>
       </c>
       <c r="K587" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
     </row>
     <row r="588" spans="1:11" x14ac:dyDescent="0.2">
@@ -37575,7 +37568,7 @@
         <v>1</v>
       </c>
       <c r="K588" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
     </row>
     <row r="589" spans="1:11" x14ac:dyDescent="0.2">
@@ -37596,7 +37589,7 @@
         <v>1</v>
       </c>
       <c r="K589" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
     </row>
     <row r="590" spans="1:11" x14ac:dyDescent="0.2">
@@ -37613,7 +37606,7 @@
         <v>41</v>
       </c>
       <c r="K590" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="591" spans="1:11" x14ac:dyDescent="0.2">
@@ -37634,7 +37627,7 @@
         <v>2</v>
       </c>
       <c r="K591" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="592" spans="1:11" x14ac:dyDescent="0.2">
@@ -37738,7 +37731,7 @@
         <v>8</v>
       </c>
       <c r="D598" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F598" s="1">
         <v>0</v>
@@ -37761,7 +37754,7 @@
         <v>41</v>
       </c>
       <c r="K599" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="600" spans="1:11" x14ac:dyDescent="0.2">
@@ -37838,7 +37831,7 @@
         <v>41</v>
       </c>
       <c r="K604" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="605" spans="1:11" x14ac:dyDescent="0.2">
@@ -37865,7 +37858,7 @@
         <v>2</v>
       </c>
       <c r="K605" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
     </row>
     <row r="606" spans="1:11" x14ac:dyDescent="0.2">
@@ -37886,7 +37879,7 @@
         <v>1</v>
       </c>
       <c r="K606" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="607" spans="1:11" x14ac:dyDescent="0.2">
@@ -37907,7 +37900,7 @@
         <v>2</v>
       </c>
       <c r="K607" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="608" spans="1:11" x14ac:dyDescent="0.2">
@@ -37921,13 +37914,13 @@
         <v>4</v>
       </c>
       <c r="D608" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J608" s="1">
         <v>2</v>
       </c>
       <c r="K608" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
     </row>
     <row r="609" spans="1:11" x14ac:dyDescent="0.2">
@@ -37944,7 +37937,7 @@
         <v>41</v>
       </c>
       <c r="K609" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
     </row>
     <row r="610" spans="1:11" x14ac:dyDescent="0.2">
@@ -37971,7 +37964,7 @@
         <v>3</v>
       </c>
       <c r="K610" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
     </row>
     <row r="611" spans="1:11" x14ac:dyDescent="0.2">
@@ -37998,7 +37991,7 @@
         <v>2</v>
       </c>
       <c r="K611" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
     </row>
     <row r="612" spans="1:11" x14ac:dyDescent="0.2">
@@ -38022,7 +38015,7 @@
         <v>8</v>
       </c>
       <c r="K612" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
     </row>
     <row r="613" spans="1:11" x14ac:dyDescent="0.2">
@@ -38046,7 +38039,7 @@
         <v>8</v>
       </c>
       <c r="K613" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
     </row>
     <row r="614" spans="1:11" x14ac:dyDescent="0.2">
@@ -38063,7 +38056,7 @@
         <v>41</v>
       </c>
       <c r="K614" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="615" spans="1:11" x14ac:dyDescent="0.2">
@@ -38137,7 +38130,7 @@
         <v>5</v>
       </c>
       <c r="D619" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F619" s="1">
         <v>0</v>
@@ -38160,7 +38153,7 @@
         <v>41</v>
       </c>
       <c r="K620" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="621" spans="1:11" x14ac:dyDescent="0.2">
@@ -38237,7 +38230,7 @@
         <v>41</v>
       </c>
       <c r="K625" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="626" spans="1:11" x14ac:dyDescent="0.2">
@@ -38326,7 +38319,7 @@
         <v>6</v>
       </c>
       <c r="D631" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F631" s="1">
         <v>0</v>
@@ -38349,7 +38342,7 @@
         <v>41</v>
       </c>
       <c r="K632" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="633" spans="1:11" x14ac:dyDescent="0.2">
@@ -38426,7 +38419,7 @@
         <v>41</v>
       </c>
       <c r="K637" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="638" spans="1:11" x14ac:dyDescent="0.2">
@@ -38467,7 +38460,7 @@
         <v>7</v>
       </c>
       <c r="K639" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="640" spans="1:11" x14ac:dyDescent="0.2">
@@ -38491,7 +38484,7 @@
         <v>9</v>
       </c>
       <c r="K640" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="641" spans="1:11" x14ac:dyDescent="0.2">
@@ -38515,7 +38508,7 @@
         <v>7</v>
       </c>
       <c r="K641" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="642" spans="1:11" x14ac:dyDescent="0.2">
@@ -38539,7 +38532,7 @@
         <v>7</v>
       </c>
       <c r="K642" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="643" spans="1:11" x14ac:dyDescent="0.2">
@@ -38563,7 +38556,7 @@
         <v>7</v>
       </c>
       <c r="K643" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="644" spans="1:11" x14ac:dyDescent="0.2">
@@ -38587,7 +38580,7 @@
         <v>7</v>
       </c>
       <c r="K644" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="645" spans="1:11" x14ac:dyDescent="0.2">
@@ -38611,7 +38604,7 @@
         <v>7</v>
       </c>
       <c r="K645" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="646" spans="1:11" x14ac:dyDescent="0.2">
@@ -38625,7 +38618,7 @@
         <v>9</v>
       </c>
       <c r="D646" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F646" s="1">
         <v>7</v>
@@ -38637,7 +38630,7 @@
         <v>12</v>
       </c>
       <c r="K646" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
     </row>
     <row r="647" spans="1:11" x14ac:dyDescent="0.2">
@@ -38654,7 +38647,7 @@
         <v>41</v>
       </c>
       <c r="K647" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="648" spans="1:11" x14ac:dyDescent="0.2">
@@ -38678,7 +38671,7 @@
         <v>7</v>
       </c>
       <c r="K648" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="649" spans="1:11" x14ac:dyDescent="0.2">
@@ -38702,7 +38695,7 @@
         <v>7</v>
       </c>
       <c r="K649" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="650" spans="1:11" x14ac:dyDescent="0.2">
@@ -38726,7 +38719,7 @@
         <v>7</v>
       </c>
       <c r="K650" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="651" spans="1:11" x14ac:dyDescent="0.2">
@@ -38750,7 +38743,7 @@
         <v>7</v>
       </c>
       <c r="K651" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
     </row>
     <row r="652" spans="1:11" x14ac:dyDescent="0.2">
@@ -38767,7 +38760,7 @@
         <v>41</v>
       </c>
       <c r="K652" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="653" spans="1:11" x14ac:dyDescent="0.2">
@@ -38856,7 +38849,7 @@
         <v>6</v>
       </c>
       <c r="D658" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F658" s="1">
         <v>0</v>
@@ -38879,7 +38872,7 @@
         <v>41</v>
       </c>
       <c r="K659" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="660" spans="1:11" x14ac:dyDescent="0.2">
@@ -38956,7 +38949,7 @@
         <v>41</v>
       </c>
       <c r="K664" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="665" spans="1:11" x14ac:dyDescent="0.2">
@@ -39062,7 +39055,7 @@
         <v>7</v>
       </c>
       <c r="D671" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F671" s="1">
         <v>0</v>
@@ -39085,7 +39078,7 @@
         <v>41</v>
       </c>
       <c r="K672" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="673" spans="1:11" x14ac:dyDescent="0.2">
@@ -39124,7 +39117,7 @@
         <v>2</v>
       </c>
       <c r="K674" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
     </row>
     <row r="675" spans="1:11" x14ac:dyDescent="0.2">
@@ -39145,7 +39138,7 @@
         <v>2</v>
       </c>
       <c r="K675" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
     </row>
     <row r="676" spans="1:11" x14ac:dyDescent="0.2">
@@ -39177,7 +39170,7 @@
         <v>41</v>
       </c>
       <c r="K677" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="678" spans="1:11" x14ac:dyDescent="0.2">
@@ -39284,7 +39277,7 @@
         <v>41</v>
       </c>
       <c r="K684" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="685" spans="1:11" x14ac:dyDescent="0.2">
@@ -39361,7 +39354,7 @@
         <v>41</v>
       </c>
       <c r="K689" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="690" spans="1:11" x14ac:dyDescent="0.2">
@@ -39437,7 +39430,7 @@
         <v>5</v>
       </c>
       <c r="D694" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F694" s="1">
         <v>0</v>
@@ -39446,7 +39439,7 @@
         <v>6</v>
       </c>
       <c r="K694" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="695" spans="1:11" x14ac:dyDescent="0.2">
@@ -39537,7 +39530,7 @@
         <v>41</v>
       </c>
       <c r="K700" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="701" spans="1:11" x14ac:dyDescent="0.2">
@@ -39600,7 +39593,7 @@
         <v>0</v>
       </c>
       <c r="K704" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
     </row>
     <row r="705" spans="1:11" x14ac:dyDescent="0.2">
@@ -39691,7 +39684,7 @@
         <v>41</v>
       </c>
       <c r="K710" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="711" spans="1:11" x14ac:dyDescent="0.2">
@@ -39712,7 +39705,7 @@
         <v>5</v>
       </c>
       <c r="K711" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="712" spans="1:11" x14ac:dyDescent="0.2">
@@ -39733,7 +39726,7 @@
         <v>5</v>
       </c>
       <c r="K712" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="713" spans="1:11" x14ac:dyDescent="0.2">
@@ -39754,7 +39747,7 @@
         <v>5</v>
       </c>
       <c r="K713" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="714" spans="1:11" x14ac:dyDescent="0.2">
@@ -39775,7 +39768,7 @@
         <v>5</v>
       </c>
       <c r="K714" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="715" spans="1:11" x14ac:dyDescent="0.2">
@@ -39796,7 +39789,7 @@
         <v>4</v>
       </c>
       <c r="K715" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="716" spans="1:11" x14ac:dyDescent="0.2">
@@ -39817,7 +39810,7 @@
         <v>4</v>
       </c>
       <c r="K716" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="717" spans="1:11" x14ac:dyDescent="0.2">
@@ -39838,7 +39831,7 @@
         <v>4</v>
       </c>
       <c r="K717" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="718" spans="1:11" x14ac:dyDescent="0.2">
@@ -39859,7 +39852,7 @@
         <v>4</v>
       </c>
       <c r="K718" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="719" spans="1:11" x14ac:dyDescent="0.2">
@@ -39873,7 +39866,7 @@
         <v>9</v>
       </c>
       <c r="D719" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F719" s="1">
         <v>4</v>
@@ -39885,7 +39878,7 @@
         <v>12</v>
       </c>
       <c r="K719" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="720" spans="1:11" x14ac:dyDescent="0.2">
@@ -39902,7 +39895,7 @@
         <v>41</v>
       </c>
       <c r="K720" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="721" spans="1:11" x14ac:dyDescent="0.2">
@@ -39923,7 +39916,7 @@
         <v>4</v>
       </c>
       <c r="K721" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="722" spans="1:11" x14ac:dyDescent="0.2">
@@ -39944,7 +39937,7 @@
         <v>4</v>
       </c>
       <c r="K722" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="723" spans="1:11" x14ac:dyDescent="0.2">
@@ -39965,7 +39958,7 @@
         <v>4</v>
       </c>
       <c r="K723" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="724" spans="1:11" x14ac:dyDescent="0.2">
@@ -39986,7 +39979,7 @@
         <v>4</v>
       </c>
       <c r="K724" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="725" spans="1:11" x14ac:dyDescent="0.2">
@@ -40003,7 +39996,7 @@
         <v>41</v>
       </c>
       <c r="K725" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="726" spans="1:11" x14ac:dyDescent="0.2">
@@ -40027,7 +40020,7 @@
         <v>1</v>
       </c>
       <c r="K726" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="727" spans="1:11" x14ac:dyDescent="0.2">
@@ -40062,7 +40055,7 @@
         <v>41</v>
       </c>
       <c r="K728" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="729" spans="1:11" x14ac:dyDescent="0.2">
@@ -40139,7 +40132,7 @@
         <v>41</v>
       </c>
       <c r="K733" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="734" spans="1:11" x14ac:dyDescent="0.2">
@@ -40273,7 +40266,7 @@
         <v>9</v>
       </c>
       <c r="D742" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F742" s="1">
         <v>0</v>
@@ -40282,7 +40275,7 @@
         <v>4</v>
       </c>
       <c r="K742" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
     </row>
     <row r="743" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
clean and tidy method for calculating the tlx factor counts
</commit_message>
<xml_diff>
--- a/data/source/i1_raw_data.xlsx
+++ b/data/source/i1_raw_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/djo/dev/au/au_diss/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3EA9D7-713F-504A-AF1E-F48398DFE83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1DE988E-8CA9-4641-BC3D-D3521D27D36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20040" yWindow="500" windowWidth="40120" windowHeight="33340" activeTab="7" xr2:uid="{9D3AC3E5-42CD-5B4C-9A6D-E91B574DC308}"/>
+    <workbookView xWindow="20040" yWindow="500" windowWidth="40120" windowHeight="33340" activeTab="1" xr2:uid="{9D3AC3E5-42CD-5B4C-9A6D-E91B574DC308}"/>
   </bookViews>
   <sheets>
     <sheet name="DEMO" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1609" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="253">
   <si>
     <t>Participant</t>
   </si>
@@ -10051,16 +10051,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46490600-6C03-4440-989B-063E2997EAC0}">
-  <dimension ref="A1:U63"/>
+  <dimension ref="A1:T63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
     <col min="2" max="5" width="4.83203125" style="1" customWidth="1"/>
     <col min="6" max="19" width="4.83203125" customWidth="1"/>
-    <col min="20" max="20" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -10118,11 +10117,8 @@
       <c r="S1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="T1" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1001</v>
       </c>
@@ -10181,7 +10177,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1003</v>
       </c>
@@ -10240,7 +10236,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>1005</v>
       </c>
@@ -10298,9 +10294,9 @@
       <c r="S4" s="1">
         <v>2</v>
       </c>
-      <c r="U4" s="1"/>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="T4" s="1"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>1006</v>
       </c>
@@ -10359,7 +10355,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>1007</v>
       </c>
@@ -10418,7 +10414,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>1008</v>
       </c>
@@ -10477,7 +10473,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>1009</v>
       </c>
@@ -10536,7 +10532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>1010</v>
       </c>
@@ -10595,7 +10591,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>1011</v>
       </c>
@@ -10654,7 +10650,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>1012</v>
       </c>
@@ -10713,7 +10709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>1013</v>
       </c>
@@ -10772,7 +10768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>1014</v>
       </c>
@@ -10831,7 +10827,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>1015</v>
       </c>
@@ -10890,7 +10886,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>1016</v>
       </c>
@@ -10949,7 +10945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>1017</v>
       </c>

</xml_diff>